<commit_message>
Fix dashboard currency handling
</commit_message>
<xml_diff>
--- a/scripts/test-fixtures/reclassify-stress-test.xlsx
+++ b/scripts/test-fixtures/reclassify-stress-test.xlsx
@@ -1074,7 +1074,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:H8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1096,6 +1096,9 @@
         <v>Tax</v>
       </c>
       <c r="G1" t="str">
+        <v>Currency</v>
+      </c>
+      <c r="H1" t="str">
         <v>Net Pay Date</v>
       </c>
     </row>
@@ -1119,6 +1122,9 @@
         <v>1480</v>
       </c>
       <c r="G2" t="str">
+        <v>USD</v>
+      </c>
+      <c r="H2" t="str">
         <v>2025-01-30</v>
       </c>
     </row>
@@ -1142,6 +1148,9 @@
         <v>1508</v>
       </c>
       <c r="G3" t="str">
+        <v>USD</v>
+      </c>
+      <c r="H3" t="str">
         <v>2025-02-30</v>
       </c>
     </row>
@@ -1165,6 +1174,9 @@
         <v>1536</v>
       </c>
       <c r="G4" t="str">
+        <v>USD</v>
+      </c>
+      <c r="H4" t="str">
         <v>2025-03-30</v>
       </c>
     </row>
@@ -1188,6 +1200,9 @@
         <v>1564</v>
       </c>
       <c r="G5" t="str">
+        <v>USD</v>
+      </c>
+      <c r="H5" t="str">
         <v>2025-04-30</v>
       </c>
     </row>
@@ -1211,6 +1226,9 @@
         <v>1592</v>
       </c>
       <c r="G6" t="str">
+        <v>USD</v>
+      </c>
+      <c r="H6" t="str">
         <v>2025-05-30</v>
       </c>
     </row>
@@ -1234,6 +1252,9 @@
         <v>1620</v>
       </c>
       <c r="G7" t="str">
+        <v>USD</v>
+      </c>
+      <c r="H7" t="str">
         <v>2025-06-30</v>
       </c>
     </row>
@@ -1257,12 +1278,15 @@
         <v>0</v>
       </c>
       <c r="G8" t="str">
+        <v>USD</v>
+      </c>
+      <c r="H8" t="str">
         <v>2025-06-15</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1692,7 +1716,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:F19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1705,9 +1729,12 @@
         <v>Amount</v>
       </c>
       <c r="D1" t="str">
+        <v>Currency</v>
+      </c>
+      <c r="E1" t="str">
         <v>Check Number</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Bank</v>
       </c>
     </row>
@@ -1718,6 +1745,9 @@
       <c r="B2" t="str">
         <v>2025-01-01</v>
       </c>
+      <c r="D2" t="str">
+        <v>PHP</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -1730,9 +1760,12 @@
         <v>1500</v>
       </c>
       <c r="D3" t="str">
+        <v>PHP</v>
+      </c>
+      <c r="E3" t="str">
         <v>PDC-202501</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>BPI</v>
       </c>
     </row>
@@ -1747,9 +1780,12 @@
         <v>1500</v>
       </c>
       <c r="D4" t="str">
+        <v>PHP</v>
+      </c>
+      <c r="E4" t="str">
         <v>PDC-202502</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>BPI</v>
       </c>
     </row>
@@ -1764,9 +1800,12 @@
         <v>1500</v>
       </c>
       <c r="D5" t="str">
+        <v>PHP</v>
+      </c>
+      <c r="E5" t="str">
         <v>PDC-202503</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" t="str">
         <v>BPI</v>
       </c>
     </row>
@@ -1781,9 +1820,12 @@
         <v>1500</v>
       </c>
       <c r="D6" t="str">
+        <v>PHP</v>
+      </c>
+      <c r="E6" t="str">
         <v>PDC-202504</v>
       </c>
-      <c r="E6" t="str">
+      <c r="F6" t="str">
         <v>BPI</v>
       </c>
     </row>
@@ -1798,9 +1840,12 @@
         <v>1500</v>
       </c>
       <c r="D7" t="str">
+        <v>PHP</v>
+      </c>
+      <c r="E7" t="str">
         <v>PDC-202505</v>
       </c>
-      <c r="E7" t="str">
+      <c r="F7" t="str">
         <v>BPI</v>
       </c>
     </row>
@@ -1815,9 +1860,12 @@
         <v>1500</v>
       </c>
       <c r="D8" t="str">
+        <v>PHP</v>
+      </c>
+      <c r="E8" t="str">
         <v>PDC-202506</v>
       </c>
-      <c r="E8" t="str">
+      <c r="F8" t="str">
         <v>BPI</v>
       </c>
     </row>
@@ -1832,9 +1880,12 @@
         <v>1500</v>
       </c>
       <c r="D9" t="str">
+        <v>PHP</v>
+      </c>
+      <c r="E9" t="str">
         <v>PDC-202507</v>
       </c>
-      <c r="E9" t="str">
+      <c r="F9" t="str">
         <v>BPI</v>
       </c>
     </row>
@@ -1849,9 +1900,12 @@
         <v>1500</v>
       </c>
       <c r="D10" t="str">
+        <v>PHP</v>
+      </c>
+      <c r="E10" t="str">
         <v>PDC-202508</v>
       </c>
-      <c r="E10" t="str">
+      <c r="F10" t="str">
         <v>BPI</v>
       </c>
     </row>
@@ -1866,9 +1920,12 @@
         <v>1500</v>
       </c>
       <c r="D11" t="str">
+        <v>PHP</v>
+      </c>
+      <c r="E11" t="str">
         <v>PDC-202509</v>
       </c>
-      <c r="E11" t="str">
+      <c r="F11" t="str">
         <v>BPI</v>
       </c>
     </row>
@@ -1883,9 +1940,12 @@
         <v>1500</v>
       </c>
       <c r="D12" t="str">
+        <v>PHP</v>
+      </c>
+      <c r="E12" t="str">
         <v>PDC-202510</v>
       </c>
-      <c r="E12" t="str">
+      <c r="F12" t="str">
         <v>BPI</v>
       </c>
     </row>
@@ -1900,9 +1960,12 @@
         <v>1500</v>
       </c>
       <c r="D13" t="str">
+        <v>PHP</v>
+      </c>
+      <c r="E13" t="str">
         <v>PDC-202511</v>
       </c>
-      <c r="E13" t="str">
+      <c r="F13" t="str">
         <v>BPI</v>
       </c>
     </row>
@@ -1917,9 +1980,12 @@
         <v>1500</v>
       </c>
       <c r="D14" t="str">
+        <v>PHP</v>
+      </c>
+      <c r="E14" t="str">
         <v>PDC-202512</v>
       </c>
-      <c r="E14" t="str">
+      <c r="F14" t="str">
         <v>BPI</v>
       </c>
     </row>
@@ -1934,9 +2000,12 @@
         <v>3000</v>
       </c>
       <c r="D15" t="str">
+        <v>PHP</v>
+      </c>
+      <c r="E15" t="str">
         <v>PDC-S1</v>
       </c>
-      <c r="E15" t="str">
+      <c r="F15" t="str">
         <v>BPI</v>
       </c>
     </row>
@@ -1951,9 +2020,12 @@
         <v>1500</v>
       </c>
       <c r="D16" t="str">
+        <v>PHP</v>
+      </c>
+      <c r="E16" t="str">
         <v>PDC-S2</v>
       </c>
-      <c r="E16" t="str">
+      <c r="F16" t="str">
         <v>BPI</v>
       </c>
     </row>
@@ -1968,9 +2040,12 @@
         <v>500</v>
       </c>
       <c r="D17" t="str">
+        <v>PHP</v>
+      </c>
+      <c r="E17" t="str">
         <v>PDC-S3</v>
       </c>
-      <c r="E17" t="str">
+      <c r="F17" t="str">
         <v>BPI</v>
       </c>
     </row>
@@ -1985,9 +2060,12 @@
         <v>250</v>
       </c>
       <c r="D18" t="str">
+        <v>PHP</v>
+      </c>
+      <c r="E18" t="str">
         <v>PDC-S4</v>
       </c>
-      <c r="E18" t="str">
+      <c r="F18" t="str">
         <v>BPI</v>
       </c>
     </row>
@@ -2002,15 +2080,18 @@
         <v>75</v>
       </c>
       <c r="D19" t="str">
+        <v>PHP</v>
+      </c>
+      <c r="E19" t="str">
         <v>PDC-S5</v>
       </c>
-      <c r="E19" t="str">
+      <c r="F19" t="str">
         <v>BPI</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>